<commit_message>
Atomic habits 2-1 to 2-10
</commit_message>
<xml_diff>
--- a/story.xlsx
+++ b/story.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\個人\Github 專案\Boyd Vocabulary\Story-reading\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66030917-99D4-411B-825F-C53932D69930}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1DB7DFB-9921-4E29-B741-3AE9AD85481E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2220" yWindow="690" windowWidth="20955" windowHeight="15090" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2220" yWindow="510" windowWidth="20955" windowHeight="15090" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="184">
   <si>
     <t>分類</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -2170,6 +2170,86 @@
   </si>
   <si>
     <t xml:space="preserve"> The two-step process to changing your identity. Your identity emerges out of your habits. You are not born with preset beliefs. Every belief, including those about yourself, is learned in condition through experience. Certainly, there are some aspects of your identity that tend to remain unchanged over time, like identifying as someone who is tall or short. But even for more fixed qualities and characteristics, whether you view them in a positive or negative light is determined by your experiences throughout life. To put it more precisely, your habits are how you embody your identity. When you make your bed each day, you embody the identity of an organized person. When you write each day, you embody the identity of a creative person. When you train each day, you embody the identity of an athletic person. The more you repeat a behavior, the more you reinforce the identity associated with that behavior. In fact, the word identity was originally derived from the Latin words Ascentias, which means Being, and Identidem, which means repeatedly. Your identity is literally your repeated beingness. Whatever your identity is right now, you only believe it because you have proof of it. If you go to church every Sunday for 20 years, you have evidence that you are religious. If you study biology for one hour every night, you have evidence that you are a student. If you go to the gym even when it's snowing, you have evidence that you are committed to fitness. The more evidence you have for a belief, the more strongly you will believe in it. For most of my early life, I didn't consider myself a writer. If you were to ask any of my high school teachers or college professors, they would tell you I was an average writer at best, certainly not a standout. When I began my writing career, I published a new article every Monday and Thursday for the first few years. As the evidence grew, so did my identity as a writer. I didn't start out as a writer. I became one through my habits. Of course, your habits are not the only actions that influence your identity, but by virtue of their frequency, they are usually the most important ones. Each experience in life modifies your self-image, but it's unlikely you would consider yourself a soccer player because you kicked the ball once or an artist because you scribbled a picture. As you repeat these actions, however, the evidence accumulates and your self-image begins to change. The effect of one-off experiences tends to fade away while the effect of habits gets reinforced with time, which means your habits contribute most of the evidence that shapes your identity. In this way, the process of building habits is actually the process of becoming yourself. This is a gradual evolution. We do not change by snapping our fingers and deciding to become someone entirely new. We change bit by bit, day by day, habit by habit. We are continually undergoing micro-evolutions of the self. Each habit is like a suggestion, hey, maybe this is who I am. If you finish a book, then perhaps you are the type of person who likes reading. If you go to the gym, then perhaps you are the type of person who likes exercise. If you practice playing the guitar, perhaps you are the type of person who likes music. Every action you take is a vote for the type of person you wish to become. No single instance will transform your beliefs, but as the votes build up, so does the evidence of your new identity. This is one reason why meaningful change does not require radical change. Small habits can make a meaningful difference by providing evidence of a new identity. And if a change is meaningful, it actually is big. That's the paradox of making small improvements. Putting this all together, you can see that habits are the path to changing your identity. The most practical way to change who you are is to change what you do. Each time you write a page, you are a writer. Each time you practice the violin, you are a musician. Each time you start a workout, you are an athlete. Each time you encourage your employees, you are a leader. Each habit not only gets results, but also teaches you something far more important to trust yourself. You start to believe you can actually accomplish these things. When the votes mount up and the evidence begins to change, the story you tell yourself begins to change as well. Of course, it works the opposite way too. Every time you choose to perform a bad habit, it's a vote for that identity. The good news is, you don't need to be perfect. In any election, there are going to be votes for both sides. You don't need a unanimous vote to win the election. You just need a majority. It doesn't matter if you cast a few votes for a bad behavior or an unproductive habit. Your goal is simply to win the majority of the time. New identities require new evidence. If you keep casting the same votes you've always cast, you're going to keep getting the same results you've always had. If nothing changes, nothing is going to change. It is a simple two-step process. One, Decide the type of person you want to be. Two, Prove it to yourself with small wins. First, decide who you want to be. This holds at any level, as an individual, as a team, as a community, as a nation. What do you want to stand for? What are your principles and values? Who do you wish to become? These are big questions, and many people aren't sure where to begin. But they do know what kind of results they want. To get six back abs, or to feel less anxious, or to double their salary. That's fine. Start there and work backward from the results you want to the type of person who could get those results. First yourself, who is the type of person that could get the outcome I want?”? Who is the type of person that could lose 40 pounds? Who is the type of person that could learn a new language? Who is the type of person that could run a successful start-up? For example, who is the type of person who could write a book? Well, it's probably someone who is consistent and reliable. So now you're focused shifts from writing a book, outcome-based, to being the type of person who is consistent and reliable, identity-based. This process can lead to beliefs like, I'm the kind of teacher who stands up for her students. I'm the kind of doctor who gives each patient the time and empathy they need. I'm the kind of manager who advocates for her employees.”. Once you have a handle on the type of person you want to be, you can begin taking small steps to reinforce your desired identity. I have a friend who lost over 100 pounds by asking yourself, what would a healthy person do? All day long, she would use this question as a guide. Would a healthy person walk or take a cab? Would a healthy person order a burrito or a salad? She figured if she acted like a healthy person long enough, eventually she would become that person. She was right. The concept of identity-based habits is our first introduction to another key theme in this book, feedback loops. Your habits shape your identity, and then your identity shapes your habits. It's a two-way street. The formation of all habits is a feedback loop. A concept we will explore in depth in the next chapter. But it is important to let your values, principles, and identity drive the loop, rather than your results. The focus should always be on becoming that type of person, not getting a particular outcome.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>James Clear – Atomic Habits-2-1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>James Clear – Atomic Habits-2-2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>James Clear – Atomic Habits-2-3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>James Clear – Atomic Habits-2-4</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>James Clear – Atomic Habits-2-5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>James Clear – Atomic Habits-2-6</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>James Clear – Atomic Habits-2-7</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>James Clear – Atomic Habits-2-8</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>James Clear – Atomic Habits-2-9</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>James Clear – Atomic Habits-2-10</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> The real reason habits matter. Identity change is the north star of habit change. The remainder of this book will provide you with step-by-step instructions on how to build better habits in yourself, your family, your team, your company, and anywhere else you wish. But the true question is, are you becoming the type of person you want to become? The first step is not what or how, but who. You need to know who you want to be. Otherwise, your quest for change is like a boat without a rudder. And that's why we're starting here. You have the power to change your beliefs about yourself. Your identity is not set in stone. You have a choice in every moment. You can choose the identity you want to reinforce today with the habits you choose today. And this brings us to the deeper purpose of this book, and the real reason habits matter. Building better habits isn't about littering your day with life hacks. It's not about flossing one, two at each night or taking a cold shower each morning or wearing the same outfit each day. It's not about achieving external measures of success, like earning more money, losing weight, or reducing stress. Certainly, habits can help you achieve all of these things. But fundamentally, they're not about having something. They're about becoming someone. Ultimately, your habits matter because they help you become the type of person you wish to be. They're the channel through which you develop your deepest beliefs about yourself. Quite literally, you become your habits. Chapter Summary There are three levels of change, outcome change, process change, and identity change. The most effective way to change your habits is to focus not on what you want to achieve, but on who you wish to become. Your identity emerges out of your habits. Your reaction is a vote for the type of person you wish to become. Becoming the best version of yourself requires you to continuously edit your beliefs and to upgrade and expand your identity. The real reason habits matter is not because they can get you better results, although they can do that, but because they can change your beliefs about yourself. Chapter 3 How to Build Better Habits in 4 Simple Steps In 1898, a psychologist named Edward Thorndeck conducted an experiment that would lay the foundation for our understanding of how habits form and the rules that guide our behavior. Thorndeck was interested in studying the behavior of animals, and he started by working with cats. He would place each cat inside a device known as a puzzle box. The box was designed so that the cat could escape through a door by some simple acts such as pulling a loop of cord, pressing a lever, or stepping on a platform. For example, one box contained a lever that, when pressed, would open a door on the side of the box. Once the door had been opened, the cat could dart out and run over to a bowl of food. Most cats wanted to escape as soon as they were placed inside the box. They would poke their nose into the corners, stick their paws through openings, and claw at loose objects. After a few minutes of exploration, the cats would happen to press the magical lever, the door would open, and they would escape. Thorndeck tracked the behavior of each cat across many trials. In the beginning, the animals moved around the box at random. But as soon as the lever had been pressed in the door open, the process of learning began. Gradually, each cat learned to associate the action of pressing the lever with the reward of escaping the box and getting to the food. After 20 to 30 trials, this behavior became so automatic and habitual that the cat could escape within a few seconds. For example, Thorndike noted, cat 12 took the following times to perform the act. 160 seconds, 30 seconds, 90 seconds, 60, 15, 28, 20, 30, 22, 11, 15, 20, 12, 10, 14, 10, 8, 8, 5, 10, 8, 6, 6, 7. During the first three trials, the cat escaped at an average of 1 and a half minutes. During the last three trials, it escaped at an average of 6.3 seconds. With practice, each cat made fewer rears and their actions became quicker and more automatic. Rather than repeat the same mistakes, the cat began to cut straight to the solution. From his studies, Thorndike described the learning process by stating, “behaviors followed by satisfying consequences tend to be repeated, and those that produce unpleasant consequences are less likely to be repeated.”. His work provides the perfect starting point for discussing how habits form in our own lives. It also provides answers to some fundamental questions like, What are habits, and why does the brain bother building them at all? Why are brain-built habits? A habit is a behavior that has been repeated enough times to become automatic. The process of habit formation begins with trial and error. Whenever you encounter a new situation in life, your brain has to make a decision. How do I respond to this? The first time you come across a problem, you're not sure how to solve it. Like Thorndeck's cat, you were just trying things out to see what works. Neurological activity in the brain is high during this period. You are carefully analyzing the situation and making conscious decisions about how to act. You are taking in tons of new information and trying to make sense of it all. The brain is busy learning the most effective course of action. Occasionally, like a cat pressing on a lever, you stumble across a solution. You're feeling anxious and you discover that going for a run calms you down, or you're mentally exhausted from long day of work and you learn that playing video games relaxes you. You're exploring, exploring, exploring, and then bam, a reward. After you stumble upon an unexpected reward.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> You alter your strategy for next time. Your brain immediately begins to catalog the events that preceded the reward. Wait a minute, that felt good. What did I do right before that? This is the feedback loop behind all human behavior. Try, fail, learn, try differently. With practice, the useless movements fade away and the useful actions get reinforced. That's a habit forming. Whenever you face a problem repeatedly, your brain begins to automate the process of solving it. Your habits are just a series of automatic solutions that solve the problems and stresses you face regularly. As behavioral scientist Jason Rea puts it, habits are, simply, reliable solutions to recurring problems in our environment. As habits are created, the level of activity in the brain decreases. You learn to lock in on the cues that predict success and tune out everything else. When a similar situation arises in the future, you know exactly what to look for. There is no longer a need to analyze every angle of a situation. Your brain skips the process of trial and error and creates a mental rule. If this, then that. These cognitive scripts can be followed automatically whenever the situation is appropriate. Now, whenever you feel stressed, you get the itch to run. Or as soon as you walk in the door from work, you grab the video game controller without thinking. A choice that once required effort is now automatic. A habit has been created. Habits are mental shortcuts learned from experience. In a sense, a habit is just a memory of the steps you previously followed to solve a problem in the past. Whenever the conditions are right, you can draw on this memory and automatically apply the same solution. The primary reason the brain remembers the past is to better predict what will work in the future. Habit formation is incredibly useful because the conscious mind is the bottleneck of the brain. It can only pay attention to one problem at a time. As a result, your brain is always working to preserve your conscious attention for whatever task is most essential. Whenever possible, the conscious mind likes to pawn off tasks to the non-conscious mind to do automatically. This is precisely what happens when a habit is formed. Habits reduce cognitive load and free up mental capacity so you can allocate your attention to other tasks. Despite their efficiency, some people still wonder about the benefits of habits. The argument might go like this. “Will habits make my life dull? I don't want to pigeonhole myself into a lifestyle I don't enjoy. Doesn't so much routine take away from the vibrancy and spontaneity of life?”? Hardly. Such questions set up a false dichotomy that make you think that you have to choose between building habits and attaining freedom. In reality, the two complement each other. Habits do not restrict freedom. They create it. In fact, the people who don't have their habits handled are often the ones with the least amount of freedom. Without good financial habits, you will always be struggling for the next dollar. Without good health habits, you will always seem to be short on energy. Without good learning habits, you will always feel like you're behind the curve. If you're always being forced to make decisions about simple tasks, when should I work out? where do I go to write? when do I pay the bills? Then you have less time for freedom. It's only by making the fundamentals of life easier that you can create the mental space needed for free thinking and creativity. Conversely, when you have your habits styled in and the basics of life are handled and done, your mind is free to focus on new challenges and master the next set of problems. Building habits in the present allows you to do more of what you want in the future. The science of how habits work. The process of building a habit can be divided into four simple steps. Q, craving, response, and reward. Readers of the Power of Habit by Charles Duhig will recognize these terms. Duhig wrote a great book, and my intention is to pick up where he left off by integrating these stages into four simple laws you can apply to build better habits in life and work. Breaking the process down into these fundamental parts can help us understand what a habit is, how it works, and how to improve it. This four-step pattern is the backbone of every habit, and your brain runs through these steps in the same order each time. First, there's the Q. The Q triggers your brain to initiate a behavior. It is a bit of information that predicts a reward, something that catches your attention. Our prehistoric ancestors were paying attention to cues that signaled the location of primary rewards like food, water, and sex. Today, we spend most of our time learning cues that predict secondary rewards like money and fame, power and status, praise and approval, love and friendship, or a sense of personal satisfaction. Of course, these pursuits also indirectly improve our odds of survival and reproduction, which is the deeper motive behind everything we do. Your mind is continuously analyzing your internal and external environment, for hints of where rewards are located. Because the Q is the first indication that we are close to a reward, it naturally leads to a craving. Cravings are the second step, and they are the motivational force behind every habit. Without some level of motivation or desire, without craving a change—, we have no reason to act. What you crave is not the habit itself, but the change in state it delivers. You do not crave smoking a cigarette, you crave the feeling of relief it provides. You are not motivated by brushing your teeth, but rather by the feeling of a clean mouth. You do not want to turn on the television, you want to be entertained. Every craving is linked to a desire to change your internal state. This is an important point that we will discuss in detail later. Cravings differ from person to person. Theory, any piece of information could trigger a craving, but in practice, people are not motivated by the same cues. For a gambler, the sound of slot machines can be a potent trigger that sparks an intense wave of desire. For someone who rarely gambles, the jingles and chimes of the casino are just background noise.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> Cues are meaningless until they are interpreted. The thoughts, feelings, and emotions of the observer are what transform a queue into a craving. The third step is the response. The response is the actual habit you perform, which can take the form of a thought or an action. Whether a response occurs depends on how motivated you are and how much friction is associated with the behavior. If a particular action requires more physical or mental effort than you are willing to expend, then you won't do it. Your response also depends on your ability. It sounds simple, but a habit can only occur if you are capable of doing it. If you want to dunk a basketball, then you can't jump high enough to reach the hoop. Well, you're out of luck. Finally, the response delivers a reward. Rewards are the end goal of every habit. The queue is about noticing the reward. The craving is about wanting the reward. The response is about obtaining the reward. We chase rewards because they serve two purposes. One, they satisfy us, and two, they teach us. The first purpose of rewards is to satisfy your craving. Yes, rewards provide benefits on their own, food and water deliver energy you need to survive. Getting a promotion brings more money and respect. Getting in shape improves your health and your dating prospects. But the more immediate benefit is that rewards satisfy your craving to eat or to gain status or to win approval. At least for a moment, rewards deliver contentment and relief from craving. Second, rewards teach us which actions are worth remembering in the future. Your brain is a reward detector. As you go about your life, your sensory nervous system is continuously monitoring which actions satisfy your desires and deliver pleasure. Feelings of pleasure and disappointment are part of the feedback mechanism that helps your brain distinguish useful actions from useless ones. Rewards close the feedback loop and complete the habit cycle. If a behavior is insufficient in any of these four stages, it will not become a habit. Eliminate the queue and your habit will never start. Reduce the craving and you won't experience enough motivation to act. Make the behavior difficult and you won't be able to do it. And if the reward fails to satisfy your desire, then you'll have no reason to do it again in the future. Without the first three steps, a behavior will not occur. Without all four, a behavior will not be repeated. We can refer to this cycle as the habit loop and you can see a graphic image of it as well as a caption describing it in detail at atomichabits.com slash media. In summary, the queue triggers a craving which motivates a response, which provides a reward, which satisfies that craving and ultimately becomes associated with the queue. Together, these four steps form a neurological feedback loop, queue craving response reward, queue craving response reward that ultimately allows you to create automatic habits. This cycle is known as the habit loop. This four step process is not something that happens occasionally, but rather is an endless feedback loop that is running and active during every moment you are alive. Even now, the brain is continually scanning the environment, predicting what will happen next, trying out different responses and learning from the results. The entire process is completed in a split second, and we use it again and again without realizing everything that has been packed into the previous moment. We can split these four steps into two phases, the problem phase and the solution phase. The problem phase includes the queue and the craving, and it is when you realize that something needs to change. The solution phase includes the response and the reward, and it is when you take action and achieve the change you desire. All behaviors driven by the desire to solve a problem. Sometimes, the problem is that you notice something good and you want to obtain it. Sometimes, the problem is that you are experiencing pain and you want to relieve it. Either way, the purpose of every habit is to solve the problems you face. Imagine walking into a dark room and flipping on the light switch. You've performed this simple habit so many times that it occurs without thinking. You proceed through all four stages in the fraction of a second. The urge to act strikes you without thinking. Here are some examples. queue your phone buzzes with a new text message. craving you want to learn the contents of the message. response you grab your phone and read the text. reward you satisfy your craving to read the message and grabbing your phone becomes associated with your phone buzzing. queue your answering emails. craving you begin to feel stressed and overwhelmed by work you want to feel in control. response you bite your nails. reward you satisfy your craving to reduce stress Biting your nails becomes associated with answering email. queue you wake up craving you want to feel alert response you drink a cup of coffee. reward you satisfy your craving to feel alert Drinking coffee becomes associated with waking up. And finally, queue you smell a doughnut shop as you walk down the street near your office craving. you begin to crave a donut response you buy a donut and eat it. reward you satisfy your craving to eat a donut buying a donut becomes associated with walking down the street near your office. By the time we become adults, we rarely notice the habits that are running our lives. Most of us never give a second thought to the fact that we tie the same shoe first each morning or unplug the toaster after each use or always change into comfortable clothes after getting home from work. After decades of mental programming, we automatically slip into these patterns of thinking and acting. The four laws of behavior change. In the following chapters, we will see time and again how the four stages of queue, craving, response and reward influence nearly everything we do each day.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> But before we do that, we need to transform these four steps into a practical framework that we can use to design good habits and eliminate bad ones. I refer to this framework as the four laws of behavior change, and it provides a simple set of rules for creating good habits and breaking bad ones. You can think of each law as a lever that influences human behavior. When the levers are in the right positions, creating good habits is effortless. When they are in the wrong positions, it is nearly impossible. Here's how you can use the four laws to create a good habit. Q. The first law. Make it obvious. Craving. The second law. Make it attractive. Response. The third law. Make it easy. Reward. The fourth law. Make it satisfying. And we can invert these laws to learn how to break a bad habit. Q. Inversion of the first law. Make it invisible. Regrading. Inversion of the second law. Make it unattractive. Response. Inversion of the third law. Make it difficult. Reward. Inversion of the fourth law. Make it unsatisfying. It would be irresponsible for me to claim that these four laws are an exhaustive framework for changing any human behavior. But I think they're close. As you will see, the four laws of behavior change applied to nearly every field from sports, to politics, art, to medicine, comedy, to management. These laws can be used no matter what challenge you are facing. There is no need for completely different strategies for each habit. Whenever you want to change your behavior, you can simply ask yourself. One. How can I make it obvious? Two. How can I make it attractive? Three. How can I make it easy? Four. How can I make it satisfying? If you have ever wondered, why don't I do what I say I'm going to do? Why don't I lose the weight or stop smoking or say for retirement or start that side business? Why do I say something is important to me but never seem to make time for it? The answers to those questions can be found somewhere in these four laws. The key to creating good habits and breaking bad ones is to understand these four fundamental laws and how to alter them to your specifications. Every goal is doomed to fail if it goes against the grain of human nature. Your habits are shaped by the systems in your life. In the chapters that follow, we will discuss these laws one by one and show how you can use them to create a system in which good habits emerge naturally and bad habits with their away. Chapter Summary A habit is a behavior that has been repeated enough times to be automatic. The ultimate purpose of habits is to solve the problems of life with as little energy and effort as possible. Any habit can be broken down into a feedback loop that involves four steps, cue, craving, response and reward. The four laws of behavior change are a simple set of rules we can use to build better habits. They are one, make it obvious, two, make it attractive, three, make it easy, and four, make it satisfying. The first law, make it obvious. Chapter 4 The man who didn't look right The psychologist Gary Klein once told me a story about a woman who attended a family gathering. She had spent years working as a paramedic and, upon arriving at the event, took one look at her father-in-law and got very concerned. I don't like the way you look, she said. Her father-in-law, who was feeling perfectly fine, jokingly replied, well, I don't like your looks either.”. No, she insisted. “You need to go to the hospital now.”. A few hours later, the man was undergoing life-saving surgery after an examination had revealed that he had a blockage to a major artery and was at immediate risk of a heart attack. Without his daughter-in-law's intuition, he could have died. What did the paramedic see? How did she predict his impending heart attack? When major arteries are obstructed, the body focuses on sending blood to critical organs and away from peripheral locations near the surface of the skin. The result is a change in the pattern of distribution of blood in the face. After many years of working with people with heart failure, the woman had unknowingly developed the ability to recognize this pattern on sight. She couldn't explain what it was that she had noticed in her father-in-law's face, but she knew something was wrong. Similar stories exist in other fields. For example, military analysts can identify which blip on a radar screen is an enemy missile, and which one is a plane from their own fleet, even though they are traveling at the same speed, flying at the same altitude, and look identical on radar in nearly every respect. During the Gulf War, Lieutenant Commander Michael Riley saved an entire battleship when he ordered a missile shot down, despite the fact that it looked exactly like the battleship’s own planes on radar. He made the right call, but even his superior officers couldn't explain how he did it. Museum curators have been known to discern the difference between an authentic piece of art and an expertly produced counterfeit, even though they can't tell you precisely which details tip them off. Experienced radiologists can look at a brain scan and predict the area where a stroke will develop before any obvious signs are visible to the untrained eye. I've even heard of hairdressers noticing whether a client is pregnant based only on the feel of her hair. The human brain is a prediction machine, it is continuously taking in your surroundings and analyzing the information it comes across. Whenever you experience something repeatedly, like a paramedic seeing the face of a heart attack patient or a military analyst seeing a missile on a radar screen, your brain begins noticing what is important, sorting through the details and highlighting the relevant cues, and cataloging that information for future use. With enough practice, you can pick up on the cues that predict certain outcomes without consciously thinking about it. Automatically, your brain encodes the lessons learned through experience. We can't always explain what it is we are learning, but learning is happening all along the way.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> And your ability to notice the relevant cues in a given situation is the foundation for every habit you have. We underestimate how much our brains and bodies can do without thinking. You do not tell your hair to grow, your heart to pump, your lungs to breathe, or your stomach to digest. And yet, your body handles all this and more on autopilot. You are much more than your conscious self. Consider hunger. How do you know when you are hungry? You don't necessarily have to see a cookie on the counter to realize that it's time to eat. Appetite and hunger are governed non-consciously. Your body has a variety of feedback loops that gradually alert you when it is time to eat again, and that track what is going on around you and within you. Cravings can arise thanks to hormones and chemicals circulating through your body. Suddenly, you're hungry even though you're not quite sure what tipped you off. This is one of the most surprising insights about our habits. You don't need to be aware of the cue for habit to begin. You can notice an opportunity and take action without dedicating conscious attention to it. This is what makes a habit useful. But it's also what makes them dangerous. As habits form, your actions come under the direction of your automatic and non-conscious mind. You fall into old patterns before you realize what's happening. Unless someone points it out, you may not notice that you cover your mouth with your hand whenever you laugh, or that you apologize before asking a question, or that you have a habit of finishing other people's sentences. And the more you repeat these patterns, the less likely you become to question what you're doing and why you're doing it. I once heard of a retail clerk who was instructed to cut up empty gift cards after customers had used up the balance on the card. One day, the clerk cached out a few customers in a row who purchased with gift cards. When the next person walked up, the clerk swiped the customer's actual credit card, picked up the scissors, and then cut it in half, entirely on autopilot, before looking up at the stunned customer and realizing what had just happened. Another woman I came across in my research was a former preschool teacher who had switched to a corporate job. Even though she was now working with adults, her old habits would kick in, and she kept asking co-workers if they had washed their hands after going to the bathroom. I also found the story of a man who had spent years working as a lifeguard, and would occasionally yell, ''walk' whenever he saw a child running. Over time, the cues that Sparker habits can become so common that they are essentially invisible. The treats on the kitchen counter, the remote control next to the couch, the phone in our blanket, are responses to these cues are so deeply encoded that it may feel like the urge to act comes from nowhere. For this reason, we must begin the process of behavior change with awareness. Before we can effectively build new habits, we need to get a handle on our current ones. This can be more challenging than it sounds, because once a habit is firmly rooted in your life, it is mostly non-conscious and automatic. If a habit remains mindless, you can't expect to improve it. As a psychologist Carl Young said, ''until you make the unconscious conscious, it will direct your life, and you will call it fate.'' The Habit Scorecard The Japanese railway system is regarded as one of the best in the world. If you ever find yourself riding a train in Tokyo, you'll notice that the conductors have a peculiar habit. As each operator runs the train, they proceed through a ritual pointing at different objects and calling out commands. When the train approaches the signal, the operator will point at it and say, ''“Signal is green.”.'' As the train pulls into and out of each station, the operator will point at the speedometer and call out the exact speed. When it's time to leave, the operator will point at the timetable and state the time. Out on the platform, other employees are performing similar actions. Before each train departs, staff members will point along the edge of the platform and declare, ''“All clear!”.'' The three details identified, pointed at and named aloud. This process, known as pointing and calling, is the safety system designed to reduce mistakes. It seems silly, but it works incredibly well. Pointing and calling reduces errors by up to 85% and cuts accidents by 30%. The MTA subway system in New York City adopted a modified version that is point only, and within two years of implementation, incidents of incorrectly berthed subways fell 57%. When I visited Japan, I saw the strategy save a woman's life. Her young son stepped onto the shinkansen, one of Japan's famous bullet trains that travel at over 200 miles per hour, just as the doors were closing. She was left outside in the platform, and jammed her arm through the door to grab him. With her arms stuck in the door, the train was about to take off, but right before it pulled away, an employee performed a safety check by pointing and calling up and down the platform. In less than five seconds, he noticed the woman and managed to stop the train from leaving. The door opened, and the woman, now in tears, ran to her son, and a minute later, the train departed safely. Pointing and calling is so effective, because it raises the level of awareness from a non-conscious habit to a more conscious level. Because the train operators must use their eyes, hands, mouth, and ears, they are more likely to notice problems before something goes wrong. My wife does something similar. Whenever we are preparing to walk out the door for a trip, she verbally calls out the most essential items in her packing list. I've got my keys, I've got my wallet, I've got my glasses, I've got my husband.”. The more automatic a behavior becomes, the less likely we are to consciously think about it. And when we've done something a thousand times before, we begin to overlook things. We assume that the next time will be just like the last. We're so used to doing what we've always done, that we don't stop to question whether it is the right thing to do it all. Many of our failures in performance are largely attributable to a lack of self-awareness. One of our greatest challenges in changing habits is maintaining awareness of what we are actually doing. This helps explain why the consequences of bad habits can sneak up on us. We need a point and call system for our own lives. That's the origin of the Habits Scorecard, which is a simple exercise you can use to become more aware of your behavior. To create your own, make a list of your daily habits.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> Here's a sample of where you might start. Wake up, turn off the alarm, check my phone, go to the bathroom, weigh myself, take a shower, and so on. Once you have a full list, look at each behavior and ask yourself, is this a good habit, a bad habit, or neutral habit? If it's a good habit, write a plus sign next to it. If it is a bad habit, write a minus sign next to it. And if it's neutral, write an equal sign. For example, the list I just mentioned might look like this. Wake up, neutral habit, turn off alarm, neutral, check my phone. Probably shouldn't do that before I get out of bed. That's negative. Go to the bathroom, neutral, weigh myself, positive, take a shower, positive, and so on. The marks you give to a particular habit will depend on your situation and your goals. For someone who is trying to lose weight, eating a bagel with peanut butter every morning might be a bad habit. For someone who's trying to bulk up and add muscle, the same behavior might be a good habit. It all depends on what you're working toward. If you're interested, you can get a template to create your own habit scorecard at atomicabits.com slash scorecard. It's worth noting that scoring your habits can be a little more complex for another reason. The labels Good Habit and Bad Habit are slightly inaccurate. There aren't really any good habits or bad habits. They're only effective habits that is effective at solving problems. All habits serve you in some way, even the bad ones, which is why you repeat them. For this exercise, categorize your habits based on how they will benefit you or hurt you in the long run. Generally speaking, Good Habits will have net positive outcomes. Bad habits will have net negative outcomes. Smoking a cigarette may reduce stress right now, that's out serving you, but it's not a healthy long-term behavior. If you're still having trouble determining how to rate a particular habit on your habit scorecard, here's a question I like to use. “Does this behavior help me become the type of person I wish to be? Does this habit cast a vote for or against my desired identity?”? Habits that reinforce your desired identity are usually good. Habits that conflict with your desired identity are usually bad. As you create your Habits Scorecard, there is no need to change anything at first. The goal is simply to know what is actually going on. Leave your thoughts and actions without judgment or internal criticism. Don't blame yourself for your faults. Don't praise yourself for your successes. If you eat a chocolate bar every morning, acknowledge it, almost as if you were watching someone else. Oh, how interesting that they would do such a thing. If you binge eat, simply notice that you are eating more calories than you should. If you waste your time online, notice that you are spending your life in a way that you do not want to. The first step to changing bad habits is to be on the lookout for them. As you feel like you need extra help, then you can try pointing and calling in your own life. Say out loud the action that you are thinking of taking and what the outcome will be. If you want to cut back on your junk food habit, but you notice yourself grabbing another cookie, say out loud, I'm about to eat this cookie, but I don't need it. Eating it will cause me to gain weight and hurt my health.”. Hearing your bad habits spoken aloud makes the consequences seem more real. It adds weight to the action rather than letting yourself mindlessly slip into an old routine. This approach is useful, even if you are simply trying to remember a task on your to-do list. Just saying out loud, “Tomorrow I need to go to the post office after lunch,”, increases the odds that you will actually do it. You are getting yourself to acknowledge the need for action, and that can make all the difference. The process of behavior change always starts with awareness. Strategies like pointing and calling and the habit scorecard are focused on getting you to recognize your habits and acknowledge the cues that trigger them, which makes it possible to respond in a way that benefits you. Chapter Summary With enough practice, your brain will pick up on the cues that predict certain outcomes without consciously thinking about it. Once our habits become automatic, we stop paying attention to what we are doing. The process of behavior change always starts with awareness. You need to be aware of your habits before you can change them. Pointing and calling raises your level of awareness from a non-conscious habit to a more conscious level by verbalizing your actions. The Habits Scorecard is a simple exercise you can use to become more aware of your behavior. Chapter 5 The Best way to Start a new Habit In 2001, researchers in Great Britain began working with 248 people to build better exercise habits over the course of two weeks. The subjects were divided into three groups. The first group was the control group. They were simply asked to track how often they exercised. The second group was the “motivation” group. They were asked not only to track their workouts, but also to read some material on the benefits of exercise. The researchers also explained to the group how exercise could reduce the risk of coronary heart disease and improve heart health. Finally, there was the third group. These subjects received the same presentation as the second group, which ensured that they had equal levels of motivation. However, they were also asked to formulate a plan for when and where they would exercise over the following week. Specifically, each member of the third group completed the following sentence. “During the next week, I will partake in at least 20 minutes of vigorous exercise on this day, at this time, in this place. In the first and second groups, 35 to 38% of people exercised at least once per week. Interestingly, the motivational presentation given to the second group seemed to have no meaningful impact on the behavior of participants as soon as they left the researchers. But 91% of the third group exercised at least once per week, more than double the normal rate. The sentence that they had filled out is what researchers refer to as an implementation intention, which is a plan you make beforehand about when and where to act. That is, how you intend to implement a particular habit.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> The cues that can trigger a habit come in a wide range of forms. The feel of your phone buzzing in your pocket, the smell of chocolate chip cookies, the sound of ambulance sirens, but the two most common cues are time and location. Implementation intentions leverage both of these cues. Broadly speaking, the format for creating an implementation intention is, when situation exercises, I will perform response-y. Examples of studies have shown that implementation intentions are effective for sticking to our goals. Whether it's writing down the exact time and date of when you will get a flu shot, or recording the time of your colonoscopy appointment, they increase the odds that people will stick with habits like recycling, studying, going to sleep early, and stopping smoking. Researchers have even found that voter turnout increases when people are forced to create implementation intentions by answering questions like, what router are you taking to the polling station? At what time are you playing to go? The bus will get you there. Other successful government programs have prompted citizens to make a clear plan to send taxes in on time, or provide directions on when and where to pay late traffic bills. The punchline is clear. People who make a specific plan for when and where they will perform a new habit are more likely to follow through. Too many people try to change their habits without these basic details figured out. We tell ourselves, I'm going to eat healthier, or I'm going to write more, but we never say when and where these habits are going to happen. We leave it up to chance and hope that we will just remember to do it, or feel motivated at the right time. An implementation intention sweeps away foggy notions like, I want to work out more, or I want to be more productive, or I should vote, and transforms them into a concrete plan of action. Many people think they lack motivation, when what they really lack is clarity. It is not always obvious when and where to take action. Many people spend their entire lives waiting for the time to be right to make an improvement. Once an implementation intention has been set, you don't have to wait for inspiration to strike. Do I write a chapter today or not? Do I meditate this morning or at lunch? When the moment of action occurs, there is no need to make a decision, simply follow your predetermined plan. The simple way to apply this strategy to your habits is to fill out this sentence. I will, behavior, at, time, in, location. For example, meditation. I will meditate for one minute at 7am in my kitchen. Or studying. I will study Spanish for 20 minutes at 6pm in my bedroom. Or exercise. I will exercise for one hour at 5pm in my local gym. Marriage. I will make my partner a cup of tea at 8am in the kitchen. If you aren't sure where to start your habit, try the first day of the week, month, or year. You are more likely to take action at those times because hope is usually higher. If we have hope, we have a reason to take action. A fresh start feels motivating. There is another benefit to implementation intentions. Being specific about what you want and how you will achieve it helps you say no to things that can derail your progress, distract your attention, and pull you off course. We often say yes to little requests because we are not clear about what we need to be doing instead. When your dreams are vague, it's easy to rationalize little exceptions all day long and never get around to the specific things you need to do to succeed. Give your habits a time and a space to live in the world. The goal is to make the time in locations so obvious that with enough repetition you get the urge to do the right thing at the right time even if you can't say why. As the writer Jason Zweeg noted, obviously you're never going to just work out without conscious thought. But like a dog salivating at a bell, maybe you start to get antsy around the time of day you normally work out. There are many ways to use implementation intentions in your life and work. My favorite approach is one I learned from Stanford professor BJ Fogg who calls it the tiny habits recipe but is the strategy that I will refer to as habit stacking. Habit stacking. A simple plan to overhaul your habits. The French philosopher Denise Diderot lived nearly his entire life in poverty but that all changed one day on 1765. Diderot's daughter was about to be married and he could not afford to pay for the wedding. Despite his lack of wealth, Diderot was well known for his role as the co-founder and writer of Encyclopedia Pidi, one of the most comprehensive encyclopedias of the time. When Catherine the Great, the Empress of Russia, heard of Diderot's financial troubles, her heart went out to him. She was a book lover and greatly enjoyed his encyclopedia. She offered to buy Diderot's personal library for a thousand pounds which is the sum equal to more than $150,000 today. Suddenly, Diderot had money to spare. With his new wealth, he not only paid for the wedding but also acquired a scarlet robe for himself. Diderot's scarlet robe was beautiful. So beautiful in fact that he immediately noticed how out of place it seemed when surrounded by his more common possessions. He wrote that there was “no more coordination, no more unity, no more beauty”, between his elegant robe and the rest of his stuff. Diderot soon felt the urge to upgrade his possessions. He replaced his rug with one from Damascus. He decorated his home with expensive sculptures. He bought a mirror to place above the mantel and a better kitchen table. He tossed aside his old straw chair for a leather one. Like falling dominoes, one purchase led to the next. Diderot's behavior is not uncommon. In fact, the tendency for one purchase to lead to another has a name, the Diderot Effect. The Diderot Effect states that obtaining a new possession often creates a spiral of consumption that leads to additional purchases. You can spot this pattern everywhere. You buy a dress and have to get shoes and earrings to match. You buy a couch and suddenly question the layout of your entire living room. You buy a toy for your child and soon find yourself purchasing all of the accessories that go with it. It is a chain reaction of purchases. Many human behaviors follow this cycle.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> You often decide what to do next based on what you have just finished doing. Going to the bathroom leads to washing and drying your hands, which reminds you that you need to put dirty towels in laundry, and so you add laundry to detergent to the shopping list, and so on. No behavior happens in isolation. Each action becomes a cue that triggers the next behavior. Alright, why is this important? Well, when it comes to building new habits, you can use the connectedness of behavior to your advantage. One of the best ways to build a new habit is to identify a current habit that you already do each day, and then stack your new behavior on top. This is what I call habit stacking. Habit stacking is a special form of an implementation intention. Rather than pairing your new habit with a particular time and location, you pair it with a current habit. This method, which again was created by B.J. Fog as part of his Tiny Habits program, can be used to design an obvious cue for nearly any habit. So the habit stacking formula is, “After current habit, I will, new habit. For example, Meditation. After I pour my cup of coffee each morning, I will meditate for one minute. Exercise. After I take off my work shoes, I will immediately change into my workout clothes. Gratitude. After I sit down to dinner, I will say one thing I'm grateful for that happened today. Marriage. After I get into bed at night, I will give my partner a kiss. Safety. After I put on my running shoes, I will text a friend or family member, where I'm running, and how long it will take. The key is to tie your desired behavior into something you already do each day. Once you have mastered this basic structure, you can begin to create larger stacks by chaining small habits together. This allows you to take advantage of the natural momentum that comes from one behavior leading into the next, like a positive version of the Diderot effect. So for example, your morning routine habit stack might look like this. One. After I pour my morning cup of coffee, I will meditate for 60 seconds. Two. After I meditate for 60 seconds, I will write my to-do list for the day. Three. After I write my to-do list for the day, I will immediately begin my first task. Or you could consider a habit stack like this in the evening. One. After I finish eating dinner, I will put my plate directly into the dishwasher. Two. After I put my dishes away, I will immediately wipe down the counter. Three. After I wipe down the counter, I will set out my coffee mug for tomorrow morning. You can also insert new behaviors into the middle of your current routines. For example, you may already have a morning routine that looks something like this. Wake up, Make my bed, Take a shower. Let's say you want to develop the habit of reading morning night. Well, you can expand your habit stack and try something like this. Wake up, Make my bed, Place a book on my pillow, Take a shower. Now, when you climb into bed each night, a book will be sitting there waiting for you to enjoy. Overall, habit stacking allows you to create a simple set of rules that guide your future behavior. It's like you always have a game plan for which action should come next. And once you get comfortable with this approach, you can develop general habit stacks to guide you whenever the situation is appropriate. So for example, exercise. When I see a set of stairs, I will take them instead of using the elevator. Or social skills. When I walk into a party, I will introduce myself to someone I don't know yet. Finances. When I want to buy something over $100, I will wait at least 24 hours before purchasing it. Healthy eating. When I serve myself a meal, I will always put veggies on my plate first. Minimalism. When I buy one new item, I will give something away. “One in, one out.”. Mood. When the phone rings, I will take one deep breath and smile before answering it. Forgetfulness. When I leave a public place, I will check the table and chairs to make sure I don't leave anything behind. No matter how you use this strategy, the secret to creating a successful habit stack is selecting the right queue to kick things off. Unlike an implementation intention, which specifically states the time and location for a given behavior, habit stacking implicitly has a time and location built into it. When and where you choose the insert to have it into your daily routine can make a big difference. If you're trying to add meditation into your morning routine, but mornings are chaotic and your kids keep running into the room, then that may be the wrong place and time to build that habit. Consider when you are most likely to be successful. Don't ask yourself to do a habit or try to build a habit stack when you're likely to be occupied with something else. Your queue should also have the same frequency as your desired habit. If you want to do a habit every day, but you stack it on top of a habit that only happens on Mondays, well then that's not a good choice. One way to find the right trigger for your habit stack is by brainstorming a list of your current habits. You can use your habit scorecard, which we created in the last chapter as a starting point. Alternatively, you can create a list of two columns. In the first column, write down the habits that you do each day without fail. For example, get out of bed, Take a shower, Brush your teeth, get dressed, Brew a cup of coffee, eat breakfast, Take the kids to school, and so on. Your list can be much longer, but you get the idea. In the second column, write down all of the things that happen to you each day without fail. For example, the sun rises, or you get a text message, the song you'are listening to ends, or the sun sets. Once you're armed with these two lists, you can begin searching for the best place to layer a new habit into your lifestyle. If you're looking for more examples and guidance on this, you can download a habit stacking template at AtomicHabits.com slash HabitsSacking. Alright, so habit stacking works best when the queue is highly specific and immediately actionable. Many people select queues that are too vague. I made this mistake myself. When I wanted to start a push-up habit, my habit stack was, when I take a break for lunch, I will do 10 push-ups.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> At first glance, this sounds reasonable, but soon I realized that the trigger was unclear. Would I do my pushups before 8 lunch? After 8 lunch? Where would I do them? After a few inconsistent days, I changed my habits back to when I close my laptop for lunch. I will do 10 pushups next to my desk. Ambiguity gone. Habits like Read More or Eat Better are worthy causes, but these goals do not provide instruction on how and when to act. You need to be specific and clear after I close the door, after I brush my teeth, after I sit down at the table. The specificity is important. The more tightly bound your new habit is to a specific queue, the better the odds are that you will notice when the time comes to act. Remember, the first law of behavior change is to make it obvious. Strategies like implementation intentions and habit stacking are among the most practical ways to create obvious cues for your habits and design a clear plan for when and where to take action. Chapter summary. The first law of behavior change is make it obvious. The two most common cues are time and location. Creating an implementation intention is a strategy you can use to pair a new habit with a specific time and location. The implementation intention formula is I will behavior at time in location. Another stacking is a strategy you can use to pair a new habit with a current habit. The habit stacking formula is after current habit I will new habit. Chapter 6. Motivation is overrated. Environment often matters more. Anne Thorndyke, a primary care physician at Massachusetts General Hospital in Boston, had a crazy idea. She believed she could improve the eating habits of thousands of hospital staff and visitors without changing their willpower or motivation in the slightest way. In fact, she didn't plan on talking to them at all. Thorndyke and her colleagues designed a six month study to alter the choice architecture of the hospital cafeteria. Originally, the refrigerators located next to the cash registers in the cafeteria were filled with only soda. The researchers added water as an option to each one. Additionally, they placed baskets of bottle water next to the food stations throughout the room. Soda was still in the primary refrigerators, but now water was an option available at all drink locations. Over the next three months, the number of soda sales at the hospital dropped by 11.4%. Meanwhile, sales of bottle water increased by 25.8%. They made similar adjustments and saw similar results with the food in the cafeteria. Nobody had said a word to anyone eating there. To see a graphical representation of the layouts in the cafeteria before and after the changes, visit AtomicHabits.com slash media. People often choose products not because of what they are, but because of where they are. If I walk into the kitchen and see a plate of cookies on the counter, I'll pick up half a dozen and start eating, even if I hadn't been thinking about them beforehand and didn't necessarily feel hungry. If the communal table at the office is always filled with doughnuts and bagels, it's going to be hard not to grab one every now and then. Your habits change depending on the room you are in and the cues in front of you. Environment is the invisible hand that shapes human behavior. Despite our unique personalities, certain behaviors tend to arise again and again under certain environmental conditions. In church, people tend to talk in whispers. On a dark street, people act wary and guarded. In this way, the most common form of change is not internal, but external. We are changed by the world around us. Every habit is context dependent. In 1936, psychologists Kurt Lewin wrote a simple equation that makes a powerful statement. Behavior is a function of the person in their environment, or B equals FPE. It didn't take long for Lewin's equation to be tested in business. In 1952, the economist Hawkins Stern described a phenomenon he called Suggestion Impulse Buying, which “is triggered when a shopper sees a product for the first time and visualizes the need for it. In other words, customers will occasionally buy products not because they want them, but because of how they are presented to them. For example, items at eye level tend to be purchased more than those down near the floor. For this reason, you'll find expensive brand names featured in easy-to-reach locations on store shelves because they drive the most profit, while cheaper alternatives are tucked away and harder to reach spots. The same goes for end caps, which are the units at the end of aisles. End caps are money-making machines for retailers because they are obvious locations that encounter a lot of foot traffic. For example, 45% of Coca-Cola sales come specifically from end of the aisle racks. The more obviously available a product or service is, the more likely you are to try it. People drink but Light because it is in every bar and visit Starbucks because it is on every corner. We like to think that we are in control. If we choose water over soda, we assume it is because we wanted to do so. The truth, however, is that many of the actions we take each day are shaped not by purposeful drive and choice, but by the most obvious option. Every living being has its own methods for sensing and understanding the world. Eagles have remarkable long-distance vision. Ox can smell by “tasting the air” with their highly sensitive tongues. Sharks can detect small amounts of electricity and vibrations in the water caused by nearby fish. Even bacteria have chemo receptors, tiny sensory cells that allow them to detect toxic chemicals in their environment. In humans, perception is directed by the sensory nervous system.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> We perceive the world through sight, sound, smell, touch, and taste. But we also have other ways of sensing stimuli. Some are conscious, but many are non-conscious. For example, you can notice when the temperature drops before a storm, or when the pain in your gut rises during a stomach ache, or when you fall off balance while walking on rocky ground. Receptors in your body pick up on a wide range of internal stimuli, such as the amount of salt in your blood or the need to drink when thirsty. The most powerful of all human sensory abilities, however, is vision. The human body has about 11 million sensory receptors. Approximately 10 million of those are dedicated to sight. Some experts estimate that half of the brain's resources are used on vision. Given that we are more dependent on vision than on any other sense, it should come as no surprise that visual cues are the greatest catalyst of our behavior. For this reason, a small change in what you see can lead to a big shift in what you do. As a result, you can imagine how important it is to live and work in environments that are filled with productive cues and devoid of unproductive ones. Thankfully, there's good news in this respect. You don't have to be the victim of your environment. You can also be the architect of it. How to design your environment for success During the energy crisis in oil embargo of the 1970s, Dutch researchers began to pay close attention to the country's energy usage. In one suburb near Amsterdam, they found that some homeowners used 30% less energy than their neighbors, despite the homes being of similar size and getting electricity for the same price. It turned out the houses in this neighborhood were nearly identical except for one feature, the location of the electrical meter. Some had one in the basement. Other houses had electrical meter upstairs in the main hallway. As you may guess, the homes with the meters located in the main hallway used less electricity. When their energy was obvious and easy to track, people changed their behavior. Every habit is initiated by a cue, and we are more likely to notice cues that stand out. Unfortunately, the environments where we live and work often make it easy to not notice or not do certain actions because there is no obvious cue to trigger the behavior. It's easy to not practice the guitar when it's tucked away in the closet. It's easy to not read a book when the bookshelf is in the corner of the guest room. It's easy to not take your vitamins with air out of sight in the pantry. When the cues that spark a habit are subtle or hidden, they are easy to ignore. By comparison, creating obvious visual cues can draw your attention toward a desired habit. In the early 1990s, the cleaning staff at Chippell Airport in Amsterdam installed a small sticker that looked like a fly near the center of each urinal. Apparently, when men stepped up to the urinals, they aimed for what they thought was a bug. The stickers improved their aim and significantly reduced “spillage” around the urinals. Further analysis determined that the stickers cut bathroom cleaning costs by 8% per year. I've experienced the power of obvious cues in my own life. I used to buy apples from the store, put them in the crisper at the bottom of the refrigerator, and forget all about them. By the time I remembered, the apples would have gone bad. I never saw them, so I never ate them. Eventually, I took my own advice and redesigned the environment. I bought a large display bowl and placed it in the middle of the kitchen counter. The next time I bought apples, that was where they went, out in the open where I could see them. Almost like magic, I began eating a few apples a day simply because they were obvious rather than out of sight. Here are a few ways you can redesign your environment and make the cues of your preferred habits more obvious. If you want to remember to take your medication each night, put your pill bottle directly next to the faucet on your bathroom counter. If you want to practice guitar more frequently, place your guitar stand in the middle of the living room. If you want to remember to send more thank you notes, keep a stack of stationery on your desk. If you want to drink more water, fill up a few water bottles each morning and place them in common locations around the house or the office. If you want to make a habit a big part of your life, then make the cue a big part of your environment. The most persistent behaviors usually have multiple cues. Consider how many different ways a smoker could be prompted to pull out a cigarette, driving the car, seeing a friend's mug, feeling stressed at work, and so on. The same strategy can be employed for good habits. By sprinkling triggers throughout your surroundings, you increase the odds that you'll think about your habit throughout the day. Make sure the best choice is the most obvious one. Making a better decision is easy and natural when the cues for good habits are right in front of you. Environment design is powerful not only because it influences how we engage with the world, but also because we rarely do it. Most people live in a world others have created for them, but you can also the spaces where you live and work to increase your exposure to positive cues and reduce your exposure to negative ones. Environment design allows you to take back control and become the architect of your life. Be the designer of your world and not merely the consumer of it. The context is the cue. The cues that trigger a habit can start out very specific, but over time, your habits become associated not with the single trigger, but with the entire context surrounding the behavior. For example, many people drink more in social situations than they would ever drink alone. The trigger is rarely a single cue, but rather the whole situation, watching your friends order drinks, hearing the music of the bar, seeing the beers on tap. We mentally assign our habits to the locations in which they occur, the home, the office, the gym. Each location develops a connection to certain habits and routines. You establish a particular relationship with the objects under desk or the items on your kitchen counter or the things in your bedroom. Our behavior is not defined by the objects in our environment, but by our relationship to them. In fact, this is a useful way to think about the influence of environment on your behavior. Stop thinking about your environment as filled with objects. Stop thinking about it as filled with relationships.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2557,7 +2637,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:J77"/>
+  <dimension ref="A1:J89"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" style="4" customWidth="1"/>
@@ -3713,6 +3793,162 @@
         <f t="shared" si="53"/>
         <v>James Clear – Atomic Habits-1-7</v>
       </c>
+    </row>
+    <row r="78" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A78" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="D78" s="12" t="str">
+        <f t="shared" ref="D78" si="54">HYPERLINK("audio\" &amp; B78 &amp; ".mp3", B78)</f>
+        <v>James Clear – Atomic Habits-2-1</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A79" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="D79" s="12" t="str">
+        <f t="shared" ref="D79:D89" si="55">HYPERLINK("audio\" &amp; B79 &amp; ".mp3", B79)</f>
+        <v>James Clear – Atomic Habits-2-2</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A80" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C80" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="D80" s="12" t="str">
+        <f t="shared" si="55"/>
+        <v>James Clear – Atomic Habits-2-3</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A81" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C81" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="D81" s="12" t="str">
+        <f t="shared" si="55"/>
+        <v>James Clear – Atomic Habits-2-4</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A82" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C82" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="D82" s="12" t="str">
+        <f t="shared" si="55"/>
+        <v>James Clear – Atomic Habits-2-5</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A83" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C83" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="D83" s="12" t="str">
+        <f t="shared" si="55"/>
+        <v>James Clear – Atomic Habits-2-6</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A84" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="C84" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="D84" s="12" t="str">
+        <f t="shared" si="55"/>
+        <v>James Clear – Atomic Habits-2-7</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A85" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="C85" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="D85" s="12" t="str">
+        <f t="shared" si="55"/>
+        <v>James Clear – Atomic Habits-2-8</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A86" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="C86" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="D86" s="12" t="str">
+        <f t="shared" si="55"/>
+        <v>James Clear – Atomic Habits-2-9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A87" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="C87" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="D87" s="12" t="str">
+        <f t="shared" si="55"/>
+        <v>James Clear – Atomic Habits-2-10</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B88" s="1"/>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B89" s="1"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:D77" xr:uid="{00000000-0001-0000-0000-000000000000}">

</xml_diff>

<commit_message>
python 模式5 / Alchemist 更新
</commit_message>
<xml_diff>
--- a/story.xlsx
+++ b/story.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github 專用\Story\Story-reading\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCE5A306-EC0B-4A83-95CC-841FF06E6B85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50447A4F-5E4C-441A-8666-10C7F41505A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="704" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="705" uniqueCount="375">
   <si>
     <t>大類</t>
   </si>
@@ -4573,6 +4573,13 @@
   </si>
   <si>
     <t>Phrase</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>On 10th February, a local woman's handbag was snatched from her while she was refuelling her car at a petrol station in Puchong Jaya.
+Dashcam footage from another car shows a motorcyclist circling the area before marking her as a target. The motorcyclist could then later be seen positioning himself before suddenly speeding towards the woman, snatching her bag away, pulling her down to the ground.
+According to the OP's Instagram post, she lost her phone, wallet, house keys, and even her car keys.
+She later uploaded the incident to her Instagram page, urging others to remain aware and cautious of their surroundings.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -4966,7 +4973,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:K176"/>
+  <dimension ref="A1:K177"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1" customWidth="1"/>
@@ -8135,6 +8142,11 @@
       <c r="E176" s="8" t="str">
         <f t="shared" si="5"/>
         <v>Essay – Implementation Intentions</v>
+      </c>
+    </row>
+    <row r="177" spans="4:4" ht="173.25" x14ac:dyDescent="0.25">
+      <c r="D177" s="3" t="s">
+        <v>374</v>
       </c>
     </row>
   </sheetData>

</xml_diff>